<commit_message>
Prepare the handoff for GitHub Copilot
Adds .github/copilot-instructions.md (read automatically by Copilot) and a
'start here' section in HANDOFF.md with the tailoring workflow and rules.
Fixes stale details in HANDOFF.md and refreshes the example outputs from
a fresh-clone run of main (all 11 sample rows correct).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R1soysbnziRQLgsTreEaWs
</commit_message>
<xml_diff>
--- a/examples/sample_suppliers_results.xlsx
+++ b/examples/sample_suppliers_results.xlsx
@@ -34,7 +34,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -58,6 +58,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
@@ -74,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -84,6 +89,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -615,7 +621,7 @@
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>CRA GST/HST Registry confirms registration on 2026-10-08 (matched name 'University of British Columbia').</t>
+          <t>CRA GST/HST Registry confirms registration on 2026-10-13 (matched name 'University of British Columbia').</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -635,7 +641,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -667,7 +673,7 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
-          <t>CRA GST/HST Registry confirms registration on 2026-10-08 (matched name 'Amazon.com.ca ULC').</t>
+          <t>CRA GST/HST Registry confirms registration on 2026-10-13 (matched name 'Amazon.com.ca ULC').</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -677,7 +683,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -734,7 +740,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -766,7 +772,7 @@
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>CRA GST/HST Registry confirms registration on 2026-10-08 (matched name 'AIRGSM PTE. LTD.'). Simplified GST/HST registrant (non-resident digital seller): GST/HST they charge is not eligible for input tax credits, so give them your GST/HST number so they don't charge it.</t>
+          <t>CRA GST/HST Registry confirms registration on 2026-10-13 (matched name 'AIRGSM PTE. LTD.'). Simplified GST/HST registrant (non-resident digital seller): GST/HST they charge is not eligible for input tax credits, so give them your GST/HST number so they don't charge it.</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -776,7 +782,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -814,7 +820,7 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -839,20 +845,24 @@
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>NOT CONFIRMED</t>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>REGISTERED - NAME NOT MATCHED</t>
         </is>
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>CRA could not match this number with name 'Wrong Name Co' on 2026-10-08. Either the number isn't registered or the legal name differs from CRA's records (CRA doesn't say which). Check the supplier's exact legal name and re-run.</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr"/>
+          <t>CRA confirms this number is registered for GST/HST on 2026-10-13 under 'AMAZON.COM.CA ULC' (name from the BC registry (OrgBook BC)), not under the name in your sheet: 'Wrong Name Co'. If 'AMAZON.COM.CA ULC' is this supplier, update your vendor record; if not, the number may belong to another business.</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>AMAZON.COM.CA ULC</t>
+        </is>
+      </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -900,7 +910,7 @@
       <c r="S8" t="inlineStr"/>
       <c r="T8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -930,14 +940,14 @@
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>NOT CONFIRMED</t>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>REGISTERED - NAME NOT MATCHED</t>
         </is>
       </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
-          <t>CRA could not match this number with name 'UBC wrong PST' on 2026-10-08. Either the number isn't registered or the legal name differs from CRA's records (CRA doesn't say which). Check the supplier's exact legal name and re-run.</t>
+          <t>CRA: this number is registered for GST/HST on 2026-10-13, but not under 'UBC wrong PST'. Confirm the number belongs to this supplier (e.g. the legal name on their invoice) before relying on it for input tax credits.</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
@@ -953,7 +963,7 @@
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -988,7 +998,7 @@
           <t>No GST/HST number provided.</t>
         </is>
       </c>
-      <c r="O10" s="6" t="inlineStr">
+      <c r="O10" s="7" t="inlineStr">
         <is>
           <t>MANUAL CHECK</t>
         </is>
@@ -1001,7 +1011,7 @@
       <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1043,7 @@
       </c>
       <c r="J11" s="3" t="inlineStr">
         <is>
-          <t>CRA GST/HST Registry confirms registration on 2026-10-08 (matched name 'Amazon.com.ca ULC').</t>
+          <t>CRA GST/HST Registry confirms registration on 2026-10-13 (matched name 'Amazon.com.ca ULC').</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
@@ -1053,7 +1063,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -1073,19 +1083,19 @@
           <t>774075766RT0001</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>REGISTERED</t>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>REGISTERED - NAME NOT MATCHED</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>CRA GST/HST Registry confirms registration on 2026-10-08 (matched name 'North American Tutors Inc.'). The name in your sheet didn't match; 'North American Tutors Inc.' is the official corporate name for this business number, so consider updating your vendor record.</t>
+          <t>CRA confirms this number is registered for GST/HST on 2026-10-13 under 'North American Tutors Inc.' (name from the federal corporations registry), not under the name in your sheet: 'NA Tutors'. If 'North American Tutors Inc.' is this supplier, update your vendor record; if not, the number may belong to another business.</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1095,7 +1105,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -1110,21 +1120,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="8" t="inlineStr">
         <is>
           <t>Supplier tax registration check</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-13</t>
         </is>
       </c>
     </row>
@@ -1141,30 +1151,35 @@
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
+          <t>REGISTERED - NAME NOT MATCHED</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
           <t>NOT REGISTERED</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>NOT CONFIRMED</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>INVALID NUMBER</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>NO NUMBER</t>
         </is>
       </c>
-      <c r="G3" s="1" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>MANUAL CHECK</t>
         </is>
       </c>
-      <c r="H3" s="1" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>ERROR</t>
         </is>
@@ -1177,24 +1192,27 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
         <v>1</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>3</v>
       </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
       <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1214,15 +1232,18 @@
         <v>0</v>
       </c>
       <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
         <v>1</v>
       </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1239,11 +1260,11 @@
         <v>0</v>
       </c>
       <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
         <v>1</v>
       </c>
-      <c r="E6" t="n">
-        <v>0</v>
-      </c>
       <c r="F6" t="n">
         <v>0</v>
       </c>
@@ -1251,6 +1272,9 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1276,9 +1300,12 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
         <v>1</v>
       </c>
-      <c r="H7" t="n">
+      <c r="I7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1309,6 +1336,9 @@
       <c r="H8" t="n">
         <v>0</v>
       </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1320,7 +1350,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Run on 2026-10-08 from sample_suppliers.xlsx. Log file: logs/tax_check_20261008_170159.log</t>
+          <t>Run on 2026-10-13 from sample_suppliers.xlsx. Log file: logs/tax_check_20261013_154228.log</t>
         </is>
       </c>
     </row>
@@ -1355,14 +1385,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GST/HST names that don't match CRA are retried with the official name from Corporations Canada's open data.</t>
+          <t>GST/HST names that don't match CRA are retried with official names: Revenu Québec's (when a QST number is given), Corporations Canada's open data, and OrgBook BC.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NOT CONFIRMED on GST/HST usually means the legal name doesn't match CRA's records; fix the name and re-run.</t>
+          <t>GST/HST numbers whose name doesn't match are still checked by number: 'REGISTERED - NAME NOT MATCHED' means the number is registered but not under the sheet's name (CRA's name is shown when known).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Handoff refresh for the next agent: current state, next steps, current example output
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01R1soysbnziRQLgsTreEaWs
</commit_message>
<xml_diff>
--- a/examples/sample_suppliers_results.xlsx
+++ b/examples/sample_suppliers_results.xlsx
@@ -1,16 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Suppliers" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tax Check Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Suppliers" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Action List" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tax Check Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Suppliers'!$A$1:$BE$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Action List'!$A$1:$O$12</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,10 +35,14 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -43,7 +51,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00104735"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -53,12 +71,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -79,18 +97,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -456,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T12"/>
+  <dimension ref="A1:BE12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -466,19 +489,56 @@
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="55" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="55" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="55" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="55" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="55" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="60" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="22" customWidth="1" min="17" max="17"/>
+    <col width="36" customWidth="1" min="18" max="18"/>
+    <col width="30" customWidth="1" min="19" max="19"/>
     <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="34" customWidth="1" min="25" max="25"/>
+    <col width="26" customWidth="1" min="26" max="26"/>
+    <col width="34" customWidth="1" min="27" max="27"/>
+    <col width="55" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="32" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+    <col width="14" customWidth="1" min="32" max="32"/>
+    <col width="18" customWidth="1" min="33" max="33"/>
+    <col width="30" customWidth="1" min="34" max="34"/>
+    <col width="50" customWidth="1" min="35" max="35"/>
+    <col width="18" customWidth="1" min="36" max="36"/>
+    <col width="32" customWidth="1" min="37" max="37"/>
+    <col width="18" customWidth="1" min="38" max="38"/>
+    <col width="14" customWidth="1" min="39" max="39"/>
+    <col width="18" customWidth="1" min="40" max="40"/>
+    <col width="30" customWidth="1" min="41" max="41"/>
+    <col width="50" customWidth="1" min="42" max="42"/>
+    <col width="18" customWidth="1" min="43" max="43"/>
+    <col width="32" customWidth="1" min="44" max="44"/>
+    <col width="18" customWidth="1" min="45" max="45"/>
+    <col width="14" customWidth="1" min="46" max="46"/>
+    <col width="18" customWidth="1" min="47" max="47"/>
+    <col width="30" customWidth="1" min="48" max="48"/>
+    <col width="50" customWidth="1" min="49" max="49"/>
+    <col width="18" customWidth="1" min="50" max="50"/>
+    <col width="32" customWidth="1" min="51" max="51"/>
+    <col width="18" customWidth="1" min="52" max="52"/>
+    <col width="14" customWidth="1" min="53" max="53"/>
+    <col width="18" customWidth="1" min="54" max="54"/>
+    <col width="30" customWidth="1" min="55" max="55"/>
+    <col width="50" customWidth="1" min="56" max="56"/>
+    <col width="12" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -517,67 +577,252 @@
           <t>Transaction Date</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Overall</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Main Issue</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Action Needed</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Other Issues</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Vendor Name Check</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Suggested Vendor Name</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Do-Not-Use Vendor</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Province Used</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>GST/HST Status</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Number Registered</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Issue</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Tax ID Problem</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Number Checked</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Date Checked</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Registered Since</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Registration End</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Status Today</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Name Accepted by CRA</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Name Source</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Registry Name</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
         <is>
           <t>GST/HST Details</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="AC1" s="2" t="inlineStr">
         <is>
           <t>QST Status</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="AD1" s="2" t="inlineStr">
+        <is>
+          <t>QST Issue</t>
+        </is>
+      </c>
+      <c r="AE1" s="2" t="inlineStr">
+        <is>
+          <t>QST Number Checked</t>
+        </is>
+      </c>
+      <c r="AF1" s="2" t="inlineStr">
+        <is>
+          <t>QST Registered Since</t>
+        </is>
+      </c>
+      <c r="AG1" s="2" t="inlineStr">
+        <is>
+          <t>QST Registration End</t>
+        </is>
+      </c>
+      <c r="AH1" s="2" t="inlineStr">
+        <is>
+          <t>QST Name on Record</t>
+        </is>
+      </c>
+      <c r="AI1" s="2" t="inlineStr">
         <is>
           <t>QST Details</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="AJ1" s="2" t="inlineStr">
         <is>
           <t>BC PST Status</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="AK1" s="2" t="inlineStr">
+        <is>
+          <t>BC PST Issue</t>
+        </is>
+      </c>
+      <c r="AL1" s="2" t="inlineStr">
+        <is>
+          <t>BC PST Number Checked</t>
+        </is>
+      </c>
+      <c r="AM1" s="2" t="inlineStr">
+        <is>
+          <t>BC PST Registered Since</t>
+        </is>
+      </c>
+      <c r="AN1" s="2" t="inlineStr">
+        <is>
+          <t>BC PST Registration End</t>
+        </is>
+      </c>
+      <c r="AO1" s="2" t="inlineStr">
+        <is>
+          <t>BC PST Name on Record</t>
+        </is>
+      </c>
+      <c r="AP1" s="2" t="inlineStr">
         <is>
           <t>BC PST Details</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="AQ1" s="2" t="inlineStr">
         <is>
           <t>SK PST Status</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="AR1" s="2" t="inlineStr">
+        <is>
+          <t>SK PST Issue</t>
+        </is>
+      </c>
+      <c r="AS1" s="2" t="inlineStr">
+        <is>
+          <t>SK PST Number Checked</t>
+        </is>
+      </c>
+      <c r="AT1" s="2" t="inlineStr">
+        <is>
+          <t>SK PST Registered Since</t>
+        </is>
+      </c>
+      <c r="AU1" s="2" t="inlineStr">
+        <is>
+          <t>SK PST Registration End</t>
+        </is>
+      </c>
+      <c r="AV1" s="2" t="inlineStr">
+        <is>
+          <t>SK PST Name on Record</t>
+        </is>
+      </c>
+      <c r="AW1" s="2" t="inlineStr">
         <is>
           <t>SK PST Details</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="AX1" s="2" t="inlineStr">
         <is>
           <t>MB RST Status</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="AY1" s="2" t="inlineStr">
+        <is>
+          <t>MB RST Issue</t>
+        </is>
+      </c>
+      <c r="AZ1" s="2" t="inlineStr">
+        <is>
+          <t>MB RST Number Checked</t>
+        </is>
+      </c>
+      <c r="BA1" s="2" t="inlineStr">
+        <is>
+          <t>MB RST Registered Since</t>
+        </is>
+      </c>
+      <c r="BB1" s="2" t="inlineStr">
+        <is>
+          <t>MB RST Registration End</t>
+        </is>
+      </c>
+      <c r="BC1" s="2" t="inlineStr">
+        <is>
+          <t>MB RST Name on Record</t>
+        </is>
+      </c>
+      <c r="BD1" s="2" t="inlineStr">
         <is>
           <t>MB RST Details</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Name on Government Record</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="BE1" s="2" t="inlineStr">
         <is>
           <t>Checked On</t>
         </is>
@@ -609,39 +854,109 @@
           <t>PST-1000-7572</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>GST/HST: Registered - vendor name differs from CRA</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>Update the vendor name to 'University of British Columbia' (the name CRA accepted).</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>GST/HST: same number as row 9 'UBC wrong PST'</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>UPDATE NAME</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>REGISTERED</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>CRA GST/HST Registry confirms registration on 2026-10-13 (matched name 'University of British Columbia').</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>Registered - vendor name differs from CRA</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>108161779RT0001</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>Active on 2026-10-19</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>Vendor name, reworded (legal part / suffix)</t>
+        </is>
+      </c>
+      <c r="AB2" s="5" t="inlineStr">
+        <is>
+          <t>Vendor name differs from CRA's records: CRA accepted 'University of British Columbia', not 'The University of British Columbia'. Update the vendor name. CRA GST/HST Registry confirms registration on 2026-10-19 (matched name 'University of British Columbia').</t>
+        </is>
+      </c>
+      <c r="AJ2" s="3" t="inlineStr">
         <is>
           <t>REGISTERED</t>
         </is>
       </c>
-      <c r="N2" s="3" t="inlineStr">
+      <c r="AK2" s="3" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>PST-1000-7572</t>
+        </is>
+      </c>
+      <c r="AP2" s="5" t="inlineStr">
         <is>
           <t>eTaxBC: PST-1000-7572 is valid for BN 108161779.</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>University of British Columbia</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+      <c r="BE2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -661,29 +976,79 @@
           <t>857305932RT0001</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>GST/HST: same number as row 7 'Wrong Name Co'</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>MATCHES</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>REGISTERED</t>
         </is>
       </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>CRA GST/HST Registry confirms registration on 2026-10-13 (matched name 'Amazon.com.ca ULC').</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Registered - name matches</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>857305932RT0001</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>Active on 2026-10-19</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
         <is>
           <t>Amazon.com.ca ULC</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>Vendor name as entered</t>
+        </is>
+      </c>
+      <c r="AB3" s="5" t="inlineStr">
+        <is>
+          <t>CRA GST/HST Registry confirms registration on 2026-10-19 (matched name 'Amazon.com.ca ULC').</t>
+        </is>
+      </c>
+      <c r="BE3" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -708,39 +1073,89 @@
           <t>1019288451 TQ 0004</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: No GST/HST number - possible number found</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Canada's Business Registries lists 'AVIENT CANADA ULC' with business number 141490367, and CRA confirms it's registered for GST/HST under that name. Confirm with the supplier that it's theirs, then add it to the vendor record (the GST/HST account is usually 141490367RT0001).</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="P4" s="6" t="inlineStr">
         <is>
           <t>NO NUMBER</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>No GST/HST number provided.</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>No number</t>
+        </is>
+      </c>
+      <c r="R4" s="7" t="inlineStr">
+        <is>
+          <t>No GST/HST number - possible number found</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>No Tax ID</t>
+        </is>
+      </c>
+      <c r="AB4" s="5" t="inlineStr">
+        <is>
+          <t>No GST/HST number provided. Possible number: Canada's Business Registries lists 'AVIENT CANADA ULC' with business number 141490367, and CRA confirms it's registered for GST/HST under that name on 2026-10-19.</t>
+        </is>
+      </c>
+      <c r="AC4" s="3" t="inlineStr">
         <is>
           <t>REGISTERED</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="AD4" s="3" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>1019288451 TQ 0004</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>2017-08-01</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="AH4" t="inlineStr">
+        <is>
+          <t>AVIENT CANADA ULC (trade name: SPARTECH PLASTIQUES)</t>
+        </is>
+      </c>
+      <c r="AI4" s="5" t="inlineStr">
         <is>
           <t>Revenu Québec: registration valid since 2017-08-01.</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>AVIENT CANADA ULC (trade name: SPARTECH PLASTIQUES)</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+      <c r="BE4" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -760,29 +1175,74 @@
           <t>751950577RT9999</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: Simplified (digital economy) registrant</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>CRA lists this supplier as a simplified GST/HST registrant (a non-resident digital seller). GST/HST they charge isn't eligible for input tax credits: give them our GST/HST number so they stop charging it.</t>
+        </is>
+      </c>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>MATCHES</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>REGISTERED</t>
         </is>
       </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>CRA GST/HST Registry confirms registration on 2026-10-13 (matched name 'AIRGSM PTE. LTD.'). Simplified GST/HST registrant (non-resident digital seller): GST/HST they charge is not eligible for input tax credits, so give them your GST/HST number so they don't charge it.</t>
-        </is>
-      </c>
-      <c r="S5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R5" s="7" t="inlineStr">
+        <is>
+          <t>Simplified (digital economy) registrant</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>751950577RT9999</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
         <is>
           <t>AIRGSM PTE. LTD.</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Vendor name as entered</t>
+        </is>
+      </c>
+      <c r="AB5" s="5" t="inlineStr">
+        <is>
+          <t>CRA GST/HST Registry confirms registration on 2026-10-19 (matched name 'AIRGSM PTE. LTD.'). Simplified GST/HST registrant (non-resident digital seller): GST/HST they charge is not eligible for input tax credits, so give them your GST/HST number so they don't charge it.</t>
+        </is>
+      </c>
+      <c r="BE5" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -802,25 +1262,59 @@
           <t>123456789RT0001</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: Tax ID typo (fails check digit)</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Correct the Tax ID in the vendor record (Fails CRA check digit (typo)).</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="P6" s="8" t="inlineStr">
         <is>
           <t>INVALID NUMBER</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>No - invalid number</t>
+        </is>
+      </c>
+      <c r="R6" s="7" t="inlineStr">
+        <is>
+          <t>Tax ID typo (fails check digit)</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Fails CRA check digit (typo)</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>123456789RT0001</t>
+        </is>
+      </c>
+      <c r="AB6" s="5" t="inlineStr">
         <is>
           <t>'123456789RT0001' fails the CRA check digit, likely a typo</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr"/>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+      <c r="BE6" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -840,29 +1334,94 @@
           <t>857305932RT0001</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: Registered under another name</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>CRA confirms this number belongs to 'AMAZON.COM.CA ULC'. If that is this supplier, update the vendor name; if not, get the correct GST/HST number from the supplier.</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>GST/HST: same number as row 3 'Amazon.com.ca ULC' (CRA accepts the number under 'Amazon.com.ca ULC'); row 11 'Amazon.com.ca ULC' (CRA accepts the number under 'Amazon.com.ca ULC')</t>
+        </is>
+      </c>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>NOT CONFIRMED</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>AMAZON.COM.CA ULC</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="P7" s="4" t="inlineStr">
         <is>
           <t>REGISTERED - NAME NOT MATCHED</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
-        <is>
-          <t>CRA confirms this number is registered for GST/HST on 2026-10-13 under 'AMAZON.COM.CA ULC' (name from the BC registry (OrgBook BC)), not under the name in your sheet: 'Wrong Name Co'. If 'AMAZON.COM.CA ULC' is this supplier, update your vendor record; if not, the number may belong to another business.</t>
-        </is>
-      </c>
-      <c r="S7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Yes - under another name</t>
+        </is>
+      </c>
+      <c r="R7" s="7" t="inlineStr">
+        <is>
+          <t>Registered under another name</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>857305932RT0001</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>Active on 2026-10-19</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
         <is>
           <t>AMAZON.COM.CA ULC</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>Canada's Business Registries</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>AMAZON.COM.CA ULC</t>
+        </is>
+      </c>
+      <c r="AB7" s="5" t="inlineStr">
+        <is>
+          <t>CRA confirms this number is registered for GST/HST on 2026-10-19 under 'AMAZON.COM.CA ULC' (name from Canada's Business Registries), not under the name in your sheet: 'Wrong Name Co'; 'Wrong Name COMPANY'. If 'AMAZON.COM.CA ULC' is this supplier, update your vendor record; if not, the number may belong to another business.</t>
+        </is>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -882,35 +1441,79 @@
           <t>1234567890TQ0001</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="6" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: No GST/HST number</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>Ask the supplier for their GST/HST number (or confirm they're a small supplier) and add it to the vendor record.</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>QST: Invalid QST number</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="P8" s="6" t="inlineStr">
         <is>
           <t>NO NUMBER</t>
         </is>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>No number</t>
+        </is>
+      </c>
+      <c r="R8" s="7" t="inlineStr">
+        <is>
+          <t>No GST/HST number</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>No Tax ID</t>
+        </is>
+      </c>
+      <c r="AB8" s="5" t="inlineStr">
         <is>
           <t>No GST/HST number provided.</t>
         </is>
       </c>
-      <c r="K8" s="5" t="inlineStr">
+      <c r="AC8" s="8" t="inlineStr">
         <is>
           <t>INVALID NUMBER</t>
         </is>
       </c>
-      <c r="L8" s="3" t="inlineStr">
+      <c r="AD8" s="7" t="inlineStr">
+        <is>
+          <t>Invalid QST number</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>1234567890TQ0001</t>
+        </is>
+      </c>
+      <c r="AI8" s="5" t="inlineStr">
         <is>
           <t>Revenu Québec says this is not a valid QST number (likely a typo).</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -935,35 +1538,94 @@
           <t>PST-1000-7573</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
+          <t>GST/HST: Registered - legal name not confirmed</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>The number is registered, but not under the vendor name. Get the legal name from the supplier (e.g. their invoice), update the vendor name and re-check.</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>BC PST: PST number doesn't match business number; GST/HST: same number as row 2 'The University of British Columbia' (CRA accepts the number under 'University of British Columbia')</t>
+        </is>
+      </c>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>NOT CONFIRMED</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="P9" s="4" t="inlineStr">
+        <is>
           <t>REGISTERED - NAME NOT MATCHED</t>
         </is>
       </c>
-      <c r="J9" s="3" t="inlineStr">
-        <is>
-          <t>CRA: this number is registered for GST/HST on 2026-10-13, but not under 'UBC wrong PST'. Confirm the number belongs to this supplier (e.g. the legal name on their invoice) before relying on it for input tax credits.</t>
-        </is>
-      </c>
-      <c r="M9" s="4" t="inlineStr">
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Yes - name not confirmed</t>
+        </is>
+      </c>
+      <c r="R9" s="6" t="inlineStr">
+        <is>
+          <t>Registered - legal name not confirmed</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>108161779RT0001</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>Active on 2026-10-19</t>
+        </is>
+      </c>
+      <c r="AB9" s="5" t="inlineStr">
+        <is>
+          <t>CRA: this number is registered for GST/HST on 2026-10-19, but not under 'UBC wrong PST'. Confirm the number belongs to this supplier (e.g. the legal name on their invoice) before relying on it for input tax credits.</t>
+        </is>
+      </c>
+      <c r="AJ9" s="6" t="inlineStr">
         <is>
           <t>NOT CONFIRMED</t>
         </is>
       </c>
-      <c r="N9" s="3" t="inlineStr">
+      <c r="AK9" s="6" t="inlineStr">
+        <is>
+          <t>PST number doesn't match business number</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>PST-1000-7573</t>
+        </is>
+      </c>
+      <c r="AP9" s="5" t="inlineStr">
         <is>
           <t>eTaxBC: no match for PST-1000-7573 with BN 108161779. The PST number is wrong, inactive, or belongs to a different business number.</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -983,35 +1645,74 @@
           <t>1234567</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: No GST/HST number</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>Ask the supplier for their GST/HST number (or confirm they're a small supplier) and add it to the vendor record.</t>
+        </is>
+      </c>
+      <c r="K10" s="5" t="inlineStr">
+        <is>
+          <t>SK PST: Manual check needed (CAPTCHA)</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>SK</t>
+        </is>
+      </c>
+      <c r="P10" s="6" t="inlineStr">
         <is>
           <t>NO NUMBER</t>
         </is>
       </c>
-      <c r="J10" s="3" t="inlineStr">
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>No number</t>
+        </is>
+      </c>
+      <c r="R10" s="7" t="inlineStr">
+        <is>
+          <t>No GST/HST number</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>No Tax ID</t>
+        </is>
+      </c>
+      <c r="AB10" s="5" t="inlineStr">
         <is>
           <t>No GST/HST number provided.</t>
         </is>
       </c>
-      <c r="O10" s="7" t="inlineStr">
+      <c r="AQ10" s="9" t="inlineStr">
         <is>
           <t>MANUAL CHECK</t>
         </is>
       </c>
-      <c r="P10" s="3" t="inlineStr">
+      <c r="AR10" s="9" t="inlineStr">
+        <is>
+          <t>Manual check needed (CAPTCHA)</t>
+        </is>
+      </c>
+      <c r="AW10" s="5" t="inlineStr">
         <is>
           <t>Saskatchewan's PST registry has a reCAPTCHA, so it needs a person: re-run with --sk-assist to tick it once and let the script do the searches, or search the business name at https://www.sets.saskatchewan.ca/rptp/portal/footer/pst-registry.</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+      <c r="BE10" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1031,39 +1732,104 @@
           <t>857305932RT0001</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>GST/HST: same number as row 7 'Wrong Name Co'</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>MATCHES</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>REGISTERED</t>
         </is>
       </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>CRA GST/HST Registry confirms registration on 2026-10-13 (matched name 'Amazon.com.ca ULC').</t>
-        </is>
-      </c>
-      <c r="Q11" s="2" t="inlineStr">
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>Registered - name matches</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>857305932RT0001</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>Active on 2026-10-19</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>Amazon.com.ca ULC</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>Vendor name as entered</t>
+        </is>
+      </c>
+      <c r="AB11" s="5" t="inlineStr">
+        <is>
+          <t>CRA GST/HST Registry confirms registration on 2026-10-19 (matched name 'Amazon.com.ca ULC').</t>
+        </is>
+      </c>
+      <c r="AX11" s="3" t="inlineStr">
         <is>
           <t>REGISTERED</t>
         </is>
       </c>
-      <c r="R11" s="3" t="inlineStr">
+      <c r="AY11" s="3" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>857305932RT0001</t>
+        </is>
+      </c>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>AMAZON.COM.CA ULC</t>
+        </is>
+      </c>
+      <c r="BD11" s="5" t="inlineStr">
         <is>
           <t>Manitoba RST registry: active registration for BN 857305932.</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>Amazon.com.ca ULC; AMAZON.COM.CA ULC</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+      <c r="BE11" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1083,33 +1849,94 @@
           <t>774075766RT0001</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>REVIEW</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr">
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: Registered under another name</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>CRA confirms this number belongs to 'North American Tutors Inc.'. If that is this supplier, update the vendor name; if not, get the correct GST/HST number from the supplier.</t>
+        </is>
+      </c>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>NOT CONFIRMED</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>North American Tutors Inc.</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
         <is>
           <t>REGISTERED - NAME NOT MATCHED</t>
         </is>
       </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>CRA confirms this number is registered for GST/HST on 2026-10-13 under 'North American Tutors Inc.' (name from the federal corporations registry), not under the name in your sheet: 'NA Tutors'. If 'North American Tutors Inc.' is this supplier, update your vendor record; if not, the number may belong to another business.</t>
-        </is>
-      </c>
-      <c r="S12" t="inlineStr">
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Yes - under another name</t>
+        </is>
+      </c>
+      <c r="R12" s="7" t="inlineStr">
+        <is>
+          <t>Registered under another name</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>774075766RT0001</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Active on 2026-10-19</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
         <is>
           <t>North American Tutors Inc.</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>Federal corporations registry</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>North American Tutors Inc.</t>
+        </is>
+      </c>
+      <c r="AB12" s="5" t="inlineStr">
+        <is>
+          <t>CRA confirms this number is registered for GST/HST on 2026-10-19 under 'North American Tutors Inc.' (name from the federal corporations registry), not under the name in your sheet: 'NA Tutors'. If 'North American Tutors Inc.' is this supplier, update your vendor record; if not, the number may belong to another business.</t>
+        </is>
+      </c>
+      <c r="BE12" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:BE12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1120,82 +1947,697 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:O12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="40" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Company Name</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Province Used</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Tax ID</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Tax ID Problem</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Main Issue</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Action Needed</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Suggested Vendor Name</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Other Issues</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>GST/HST Status</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>QST Status</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>BC PST Status</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>SK PST Status</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>MB RST Status</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Sheet Row</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Wrong Name Co</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>857305932RT0001</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="F2" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: Registered under another name</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>CRA confirms this number belongs to 'AMAZON.COM.CA ULC'. If that is this supplier, update the vendor name; if not, get the correct GST/HST number from the supplier.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>AMAZON.COM.CA ULC</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>GST/HST: same number as row 3 'Amazon.com.ca ULC' (CRA accepts the number under 'Amazon.com.ca ULC'); row 11 'Amazon.com.ca ULC' (CRA accepts the number under 'Amazon.com.ca ULC')</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>REGISTERED - NAME NOT MATCHED</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NA Tutors</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>774075766RT0001</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: Registered under another name</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>CRA confirms this number belongs to 'North American Tutors Inc.'. If that is this supplier, update the vendor name; if not, get the correct GST/HST number from the supplier.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>North American Tutors Inc.</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>REGISTERED - NAME NOT MATCHED</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bad QST Ltee</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>No Tax ID</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: No GST/HST number</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Ask the supplier for their GST/HST number (or confirm they're a small supplier) and add it to the vendor record.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>QST: Invalid QST number</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>NO NUMBER</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>INVALID NUMBER</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Prairie Example Ltd</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SK</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>No Tax ID</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: No GST/HST number</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Ask the supplier for their GST/HST number (or confirm they're a small supplier) and add it to the vendor record.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>SK PST: Manual check needed (CAPTCHA)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>NO NUMBER</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>MANUAL CHECK</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Avient Canada ULC</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>QC</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>No Tax ID</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: No GST/HST number - possible number found</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Canada's Business Registries lists 'AVIENT CANADA ULC' with business number 141490367, and CRA confirms it's registered for GST/HST under that name. Confirm with the supplier that it's theirs, then add it to the vendor record (the GST/HST account is usually 141490367RT0001).</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>NO NUMBER</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>REGISTERED</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Typo Supplies Inc</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>123456789RT0001</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Fails CRA check digit (typo)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: Tax ID typo (fails check digit)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Correct the Tax ID in the vendor record (Fails CRA check digit (typo)).</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>INVALID NUMBER</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AIRGSM PTE. LTD.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>751950577RT9999</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>GST/HST: Simplified (digital economy) registrant</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>CRA lists this supplier as a simplified GST/HST registrant (a non-resident digital seller). GST/HST they charge isn't eligible for input tax credits: give them our GST/HST number so they stop charging it.</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>REGISTERED</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>UBC wrong PST</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>108161779RT0001</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>GST/HST: Registered - legal name not confirmed</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>The number is registered, but not under the vendor name. Get the legal name from the supplier (e.g. their invoice), update the vendor name and re-check.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>BC PST: PST number doesn't match business number; GST/HST: same number as row 2 'The University of British Columbia' (CRA accepts the number under 'University of British Columbia')</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>REGISTERED - NAME NOT MATCHED</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>NOT CONFIRMED</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>The University of British Columbia</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BC</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>10816 1779 RT0001</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>GST/HST: Registered - vendor name differs from CRA</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>Update the vendor name to 'University of British Columbia' (the name CRA accepted).</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>University of British Columbia</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>GST/HST: same number as row 9 'UBC wrong PST'</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>REGISTERED</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>REGISTERED</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Amazon.com.ca ULC</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>857305932RT0001</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>GST/HST: same number as row 7 'Wrong Name Co'</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>REGISTERED</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Amazon.com.ca ULC</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MB</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>857305932RT0001</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>GST/HST: same number as row 7 'Wrong Name Co'</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>REGISTERED</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>REGISTERED</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:O12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="90" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Supplier tax registration check</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-    </row>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Tax</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="inlineStr">
-        <is>
-          <t>REGISTERED</t>
-        </is>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>REGISTERED - NAME NOT MATCHED</t>
-        </is>
-      </c>
-      <c r="D3" s="1" t="inlineStr">
-        <is>
-          <t>NOT REGISTERED</t>
-        </is>
-      </c>
-      <c r="E3" s="1" t="inlineStr">
-        <is>
-          <t>NOT CONFIRMED</t>
-        </is>
-      </c>
-      <c r="F3" s="1" t="inlineStr">
-        <is>
-          <t>INVALID NUMBER</t>
-        </is>
-      </c>
-      <c r="G3" s="1" t="inlineStr">
-        <is>
-          <t>NO NUMBER</t>
-        </is>
-      </c>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t>MANUAL CHECK</t>
-        </is>
-      </c>
-      <c r="I3" s="1" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+      <c r="A3" s="11" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>REVIEW</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>NOT APPLICABLE</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="F3" s="11" t="inlineStr">
+        <is>
+          <t>NOT CHECKED</t>
+        </is>
+      </c>
+      <c r="G3" s="11" t="inlineStr">
+        <is>
+          <t>Rows checked</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GST/HST</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -1204,195 +2646,706 @@
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>3</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>QST</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-    </row>
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5"/>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>BC PST</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
-        <v>0</v>
+      <c r="A6" s="11" t="inlineStr">
+        <is>
+          <t>Vendor Name Check</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>MATCHES</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>UPDATE NAME</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>NOT CONFIRMED</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SK PST</t>
+          <t>Suppliers</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MB RST</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
+          <t>MATCHES: the vendor name is the name CRA has. UPDATE NAME: registration confirmed, but under the name in 'Suggested Vendor Name'; correct the vendor record. NOT CONFIRMED: CRA accepted no name we have; get the legal name from the supplier (e.g. their invoice).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Registration dates: QST dates come from Revenu Québec; GST/HST dates from CRA's simplified list, or by asking the CRA registry about specific days (the registry gives no dates itself). 'Registration End' is when a registration was cancelled; 'Active on &lt;date&gt;' means still registered that day. Registrations don't expire. Manitoba, BC and Saskatchewan's registries don't give dates.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10"/>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Run on 2026-10-13 from sample_suppliers.xlsx. Log file: logs/tax_check_20261013_154228.log</t>
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Issues by tax</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Suppliers</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>What to do</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GST/HST: CRA GST/HST Registry, plus CRA's simplified GST/HST registrant list.</t>
+          <t>GST/HST</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Same GST/HST number as another vendor</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>5</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Check whether these vendor records are the same business (a duplicate, or a trade name) or whether one of them has the wrong GST/HST number; see 'Other Issues' for the other vendor.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>QST: Revenu Québec QST validation API (TQ numbers) and Revenu Québec's NR registrant list.</t>
-        </is>
+          <t>GST/HST</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Registered - name matches</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BC PST: eTaxBC PST Number Verification Service. MB RST: Manitoba TAXcess RST Registration Registry.</t>
+          <t>GST/HST</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Registered under another name</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CRA confirms the number under the name in 'Suggested Vendor Name'. If that is this supplier, update the vendor name; if not, get the correct GST/HST number from the supplier.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SK PST: SETS PST On-Line Registry (needs --sk-assist, because of its CAPTCHA).</t>
+          <t>GST/HST</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>No GST/HST number</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Ask the supplier for their GST/HST number (or confirm they're a small supplier) and add it to the vendor record.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GST/HST names that don't match CRA are retried with official names: Revenu Québec's (when a QST number is given), Corporations Canada's open data, and OrgBook BC.</t>
+          <t>GST/HST</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Registered - vendor name differs from CRA</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Update the vendor name to the name in 'Suggested Vendor Name' (the name CRA accepted).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>GST/HST</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>No GST/HST number - possible number found</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>A business registered under exactly the vendor's name has a GST/HST number CRA confirms ('GST/HST Details'). Confirm with the supplier that it's theirs, then add it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>GST/HST</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Simplified (digital economy) registrant</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>GST/HST these suppliers charge isn't eligible for input tax credits: give them our GST/HST number so they stop charging it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>GST/HST</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Tax ID typo (fails check digit)</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Correct the Tax ID in the vendor record (a digit is wrong).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>GST/HST</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Registered - legal name not confirmed</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>The number is registered, but not under the vendor name. Get the legal name from the supplier (e.g. their invoice), update the vendor name and re-check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>QST</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>QST</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Invalid QST number</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Correct the QST number.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>BC PST</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>BC PST</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>PST number doesn't match business number</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Confirm the BC PST number and GST/HST number with the supplier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>SK PST</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Manual check needed (CAPTCHA)</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Re-run with --sk-assist (tick the CAPTCHA once) or search the name on Saskatchewan's PST registry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>MB RST</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Registered</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Status by tax</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>REGISTERED</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>REGISTERED - NAME NOT MATCHED</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>NOT REGISTERED</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="inlineStr">
+        <is>
+          <t>NOT CONFIRMED</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="inlineStr">
+        <is>
+          <t>INVALID NUMBER</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>NO NUMBER</t>
+        </is>
+      </c>
+      <c r="H28" s="11" t="inlineStr">
+        <is>
+          <t>MANUAL CHECK</t>
+        </is>
+      </c>
+      <c r="I28" s="11" t="inlineStr">
+        <is>
+          <t>ERROR</t>
+        </is>
+      </c>
+      <c r="J28" s="11" t="inlineStr">
+        <is>
+          <t>NOT APPLICABLE</t>
+        </is>
+      </c>
+      <c r="K28" s="11" t="inlineStr">
+        <is>
+          <t>NOT LOOKED UP</t>
+        </is>
+      </c>
+      <c r="L28" s="11" t="inlineStr">
+        <is>
+          <t>NOT CHECKED</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>GST/HST</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="n">
+        <v>3</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>QST</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>BC PST</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SK PST</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>MB RST</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Taxes checked in this run: GST/HST, QST, BC PST, Manitoba RST, Saskatchewan PST.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>GST/HST registration dates: checked whether each supplier is still registered today, with the cancellation date if not.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Run on 2026-10-19 from sample_suppliers.xlsx. Log file: logs/tax_check_20261019_214956.log</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>GST/HST: CRA GST/HST Registry, plus CRA's simplified GST/HST registrant list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>QST: Revenu Québec QST validation API (TQ numbers) and Revenu Québec's NR registrant list.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>BC PST: eTaxBC PST Number Verification Service. MB RST: Manitoba TAXcess RST Registration Registry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SK PST: SETS PST On-Line Registry, searched in a browser window after a person ticks its CAPTCHA once (--sk-assist, or Y in the menu); otherwise a manual check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>GST/HST names that don't match CRA are retried with official names: Revenu Québec's (when a QST number is given), Corporations Canada's open data, Canada's Business Registries (provincial companies) and OrgBook BC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
           <t>GST/HST numbers whose name doesn't match are still checked by number: 'REGISTERED - NAME NOT MATCHED' means the number is registered but not under the sheet's name (CRA's name is shown when known).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Progress file (one line per supplier, used by --resume): logs/progress_20261019_214956.csv</t>
         </is>
       </c>
     </row>

</xml_diff>